<commit_message>
Refresh Canadian Tire data and categorized list (732); add per-capita chart
</commit_message>
<xml_diff>
--- a/public/sheets/canadian-tire-stores.xlsx
+++ b/public/sheets/canadian-tire-stores.xlsx
@@ -10534,38 +10534,38 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1" t="n">
+    <row r="66" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="3" t="n">
         <v>608</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="C66" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="D66" s="1" t="s">
+      <c r="D66" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="E66" s="1" t="s">
+      <c r="E66" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="F66" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="G66" s="1" t="s">
+      <c r="G66" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="H66" s="1" t="n">
+      <c r="H66" s="3" t="n">
         <v>49.235016</v>
       </c>
-      <c r="I66" s="1" t="n">
+      <c r="I66" s="3" t="n">
         <v>-122.860456</v>
       </c>
-      <c r="J66" s="1" t="s">
+      <c r="J66" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="K66" s="1" t="s">
+      <c r="K66" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -15431,7 +15431,7 @@
         <v>1063</v>
       </c>
       <c r="K205" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20019,38 +20019,38 @@
         <v>23</v>
       </c>
     </row>
-    <row r="337" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A337" s="1" t="n">
+    <row r="337" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A337" s="3" t="n">
         <v>97</v>
       </c>
-      <c r="B337" s="1" t="s">
+      <c r="B337" s="3" t="s">
         <v>1734</v>
       </c>
-      <c r="C337" s="1" t="s">
+      <c r="C337" s="3" t="s">
         <v>1735</v>
       </c>
-      <c r="D337" s="1" t="s">
+      <c r="D337" s="3" t="s">
         <v>1734</v>
       </c>
-      <c r="E337" s="1" t="s">
+      <c r="E337" s="3" t="s">
         <v>953</v>
       </c>
-      <c r="F337" s="1" t="s">
+      <c r="F337" s="3" t="s">
         <v>1736</v>
       </c>
-      <c r="G337" s="1" t="s">
+      <c r="G337" s="3" t="s">
         <v>1737</v>
       </c>
-      <c r="H337" s="1" t="n">
+      <c r="H337" s="3" t="n">
         <v>42.847527</v>
       </c>
-      <c r="I337" s="1" t="n">
+      <c r="I337" s="3" t="n">
         <v>-80.291736</v>
       </c>
-      <c r="J337" s="1" t="s">
+      <c r="J337" s="3" t="s">
         <v>1738</v>
       </c>
-      <c r="K337" s="1" t="s">
+      <c r="K337" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -21664,38 +21664,38 @@
         <v>23</v>
       </c>
     </row>
-    <row r="384" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A384" s="1" t="n">
+    <row r="384" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A384" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B384" s="1" t="s">
+      <c r="B384" s="3" t="s">
         <v>1975</v>
       </c>
-      <c r="C384" s="1" t="s">
+      <c r="C384" s="3" t="s">
         <v>1976</v>
       </c>
-      <c r="D384" s="1" t="s">
+      <c r="D384" s="3" t="s">
         <v>1975</v>
       </c>
-      <c r="E384" s="1" t="s">
+      <c r="E384" s="3" t="s">
         <v>1977</v>
       </c>
-      <c r="F384" s="1" t="s">
+      <c r="F384" s="3" t="s">
         <v>1978</v>
       </c>
-      <c r="G384" s="1" t="s">
+      <c r="G384" s="3" t="s">
         <v>1979</v>
       </c>
-      <c r="H384" s="1" t="n">
+      <c r="H384" s="3" t="n">
         <v>46.269094</v>
       </c>
-      <c r="I384" s="1" t="n">
+      <c r="I384" s="3" t="n">
         <v>-63.145017</v>
       </c>
-      <c r="J384" s="1" t="s">
+      <c r="J384" s="3" t="s">
         <v>1980</v>
       </c>
-      <c r="K384" s="1" t="s">
+      <c r="K384" s="3" t="s">
         <v>23</v>
       </c>
     </row>
@@ -24079,39 +24079,39 @@
         <v>23</v>
       </c>
     </row>
-    <row r="453" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A453" s="1" t="n">
+    <row r="453" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A453" s="3" t="n">
         <v>320</v>
       </c>
-      <c r="B453" s="1" t="s">
+      <c r="B453" s="3" t="s">
         <v>2332</v>
       </c>
-      <c r="C453" s="1" t="s">
+      <c r="C453" s="3" t="s">
         <v>2333</v>
       </c>
-      <c r="D453" s="1" t="s">
+      <c r="D453" s="3" t="s">
         <v>2332</v>
       </c>
-      <c r="E453" s="1" t="s">
+      <c r="E453" s="3" t="s">
         <v>1988</v>
       </c>
-      <c r="F453" s="1" t="s">
+      <c r="F453" s="3" t="s">
         <v>2334</v>
       </c>
-      <c r="G453" s="1" t="s">
+      <c r="G453" s="3" t="s">
         <v>2335</v>
       </c>
-      <c r="H453" s="1" t="n">
+      <c r="H453" s="3" t="n">
         <v>48.46837</v>
       </c>
-      <c r="I453" s="1" t="n">
+      <c r="I453" s="3" t="n">
         <v>-68.514261</v>
       </c>
-      <c r="J453" s="1" t="s">
+      <c r="J453" s="3" t="s">
         <v>2336</v>
       </c>
-      <c r="K453" s="1" t="s">
-        <v>17</v>
+      <c r="K453" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="454" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>